<commit_message>
Corrida | SFE-SUPT | 2026-06-17 11:33:43.15848
</commit_message>
<xml_diff>
--- a/indicadores/SFE-SUPT_out.xlsx
+++ b/indicadores/SFE-SUPT_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="344">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="346">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -23,7 +23,7 @@
     <t xml:space="preserve">Título</t>
   </si>
   <si>
-    <t xml:space="preserve">Superficie cubierta autorizada en el total de la provincia</t>
+    <t xml:space="preserve">Superficie cubierta autorizada</t>
   </si>
   <si>
     <t xml:space="preserve">Unidad de medida</t>
@@ -74,6 +74,12 @@
     <t xml:space="preserve">const</t>
   </si>
   <si>
+    <t xml:space="preserve">Alcance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provincia de Santa Fe</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumen del correlograma</t>
   </si>
   <si>
@@ -107,13 +113,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">01/06/2026</t>
+    <t xml:space="preserve">17/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">ysonder</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -1548,9 +1554,13 @@
       <c r="J6" s="1"/>
     </row>
     <row r="7">
-      <c r="A7"/>
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
       <c r="B7"/>
-      <c r="C7"/>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7"/>
@@ -1561,7 +1571,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B8"/>
       <c r="C8"/>
@@ -1575,7 +1585,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B9"/>
       <c r="C9"/>
@@ -1591,7 +1601,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
@@ -1619,7 +1629,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
@@ -1633,7 +1643,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B13"/>
       <c r="C13"/>
@@ -1661,7 +1671,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
@@ -1675,7 +1685,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B16"/>
       <c r="C16"/>
@@ -1689,7 +1699,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -1703,7 +1713,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
@@ -1719,7 +1729,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -1733,7 +1743,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B20"/>
       <c r="C20"/>
@@ -1881,10 +1891,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C32"/>
       <c r="D32"/>
@@ -1897,10 +1907,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B33" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C33"/>
       <c r="D33"/>
@@ -1924,66 +1934,66 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="I1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="K1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="M1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="N1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="O1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="P1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="Q1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="R1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="S1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>112.834</v>
@@ -2036,7 +2046,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>110.529</v>
@@ -2093,7 +2103,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>119.058</v>
@@ -2150,7 +2160,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>145.67</v>
@@ -2207,7 +2217,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>165.803</v>
@@ -2264,7 +2274,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>181.662</v>
@@ -2321,7 +2331,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>269.554</v>
@@ -2378,7 +2388,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>186.686</v>
@@ -2435,7 +2445,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>173.524</v>
@@ -2492,7 +2502,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>138.463</v>
@@ -2549,7 +2559,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>158.218</v>
@@ -2606,7 +2616,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>188.881</v>
@@ -2663,7 +2673,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>114.267</v>
@@ -2722,7 +2732,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>130.648</v>
@@ -2781,7 +2791,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>169.106</v>
@@ -2840,7 +2850,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>139.13</v>
@@ -2899,7 +2909,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>203.308</v>
@@ -2958,7 +2968,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>151.484</v>
@@ -3017,7 +3027,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>163.351</v>
@@ -3076,7 +3086,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>305.884</v>
@@ -3135,7 +3145,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>211.78</v>
@@ -3194,7 +3204,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>180.558</v>
@@ -3253,7 +3263,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>199.105</v>
@@ -3312,7 +3322,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>175.825</v>
@@ -3371,7 +3381,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>146.122</v>
@@ -3430,7 +3440,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>139.4</v>
@@ -3489,7 +3499,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>132.99</v>
@@ -3548,7 +3558,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>149.544</v>
@@ -3607,7 +3617,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>203.211</v>
@@ -3666,7 +3676,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>184.724</v>
@@ -3725,7 +3735,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>189.677</v>
@@ -3784,7 +3794,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>236.141</v>
@@ -3843,7 +3853,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>134.451</v>
@@ -3902,7 +3912,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>159.811</v>
@@ -3961,7 +3971,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>153.489</v>
@@ -4020,7 +4030,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>127.706</v>
@@ -4079,7 +4089,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>195.114</v>
@@ -4138,7 +4148,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>109.513</v>
@@ -4197,7 +4207,7 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>198.145</v>
@@ -4256,7 +4266,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>179.981</v>
@@ -4315,7 +4325,7 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>236.16</v>
@@ -4374,7 +4384,7 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>168.132</v>
@@ -4433,7 +4443,7 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>211.493</v>
@@ -4492,7 +4502,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>174.413</v>
@@ -4551,7 +4561,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>170.252</v>
@@ -4610,7 +4620,7 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>188.387</v>
@@ -4669,7 +4679,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>181.598</v>
@@ -4728,7 +4738,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>169.577</v>
@@ -4787,7 +4797,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>131.562</v>
@@ -4846,7 +4856,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B51" s="2" t="n">
         <v>135.388</v>
@@ -4905,7 +4915,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>164.243</v>
@@ -4964,7 +4974,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>169.864</v>
@@ -5023,7 +5033,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>191.431</v>
@@ -5082,7 +5092,7 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>144.59</v>
@@ -5141,7 +5151,7 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>201.408</v>
@@ -5200,7 +5210,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B57" s="2" t="n">
         <v>140.873</v>
@@ -5259,7 +5269,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B58" s="2" t="n">
         <v>162.092</v>
@@ -5318,7 +5328,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B59" s="2" t="n">
         <v>200.378</v>
@@ -5377,7 +5387,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B60" s="2" t="n">
         <v>150.052</v>
@@ -5436,7 +5446,7 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B61" s="2" t="n">
         <v>165.738</v>
@@ -5495,7 +5505,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B62" s="2" t="n">
         <v>148.733</v>
@@ -5554,7 +5564,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B63" s="2" t="n">
         <v>151.61</v>
@@ -5613,7 +5623,7 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>146.369</v>
@@ -5672,7 +5682,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B65" s="2" t="n">
         <v>144.377</v>
@@ -5731,7 +5741,7 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>235.468</v>
@@ -5790,7 +5800,7 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B67" s="2" t="n">
         <v>167.592</v>
@@ -5849,7 +5859,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B68" s="2" t="n">
         <v>180.213</v>
@@ -5908,7 +5918,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B69" s="2" t="n">
         <v>166.706</v>
@@ -5967,7 +5977,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B70" s="2" t="n">
         <v>165.325</v>
@@ -6026,7 +6036,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B71" s="2" t="n">
         <v>201.002</v>
@@ -6085,7 +6095,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B72" s="2" t="n">
         <v>144.715</v>
@@ -6144,7 +6154,7 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B73" s="2" t="n">
         <v>131.797</v>
@@ -6203,7 +6213,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B74" s="2" t="n">
         <v>145.07</v>
@@ -6262,7 +6272,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B75" s="2" t="n">
         <v>113.21</v>
@@ -6321,7 +6331,7 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B76" s="2" t="n">
         <v>213.115</v>
@@ -6380,7 +6390,7 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B77" s="2" t="n">
         <v>135.498</v>
@@ -6439,7 +6449,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B78" s="2" t="n">
         <v>150.144</v>
@@ -6498,7 +6508,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B79" s="2" t="n">
         <v>209.17</v>
@@ -6557,7 +6567,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B80" s="2" t="n">
         <v>126.981</v>
@@ -6616,7 +6626,7 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B81" s="2" t="n">
         <v>167.156</v>
@@ -6675,7 +6685,7 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B82" s="2" t="n">
         <v>125.343</v>
@@ -6734,7 +6744,7 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B83" s="2" t="n">
         <v>128.517</v>
@@ -6793,7 +6803,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B84" s="2" t="n">
         <v>147.469</v>
@@ -6852,7 +6862,7 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B85" s="2" t="n">
         <v>193.647</v>
@@ -6911,7 +6921,7 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B86" s="2" t="n">
         <v>165.361</v>
@@ -6970,7 +6980,7 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B87" s="2" t="n">
         <v>124.194</v>
@@ -7029,7 +7039,7 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B88" s="2" t="n">
         <v>222.618</v>
@@ -7088,7 +7098,7 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B89" s="2" t="n">
         <v>172.57</v>
@@ -7147,7 +7157,7 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B90" s="2" t="n">
         <v>170.245</v>
@@ -7206,7 +7216,7 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B91" s="2" t="n">
         <v>162.832</v>
@@ -7265,7 +7275,7 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B92" s="2" t="n">
         <v>197.038</v>
@@ -7324,7 +7334,7 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B93" s="2" t="n">
         <v>186.336</v>
@@ -7383,7 +7393,7 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B94" s="2" t="n">
         <v>204.215</v>
@@ -7442,7 +7452,7 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B95" s="2" t="n">
         <v>156.854</v>
@@ -7501,7 +7511,7 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B96" s="2" t="n">
         <v>184.547</v>
@@ -7560,7 +7570,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B97" s="2" t="n">
         <v>151.292</v>
@@ -7619,7 +7629,7 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B98" s="2" t="n">
         <v>162.799</v>
@@ -7678,7 +7688,7 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B99" s="2" t="n">
         <v>201.706</v>
@@ -7737,7 +7747,7 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B100" s="2" t="n">
         <v>181.407</v>
@@ -7796,7 +7806,7 @@
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B101" s="2" t="n">
         <v>158.041</v>
@@ -7855,7 +7865,7 @@
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B102" s="2" t="n">
         <v>190.207</v>
@@ -7914,7 +7924,7 @@
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B103" s="2" t="n">
         <v>173.199</v>
@@ -7973,7 +7983,7 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B104" s="2" t="n">
         <v>162.015</v>
@@ -8032,7 +8042,7 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B105" s="2" t="n">
         <v>159.531</v>
@@ -8091,7 +8101,7 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B106" s="2" t="n">
         <v>159.501</v>
@@ -8150,7 +8160,7 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B107" s="2" t="n">
         <v>154.404</v>
@@ -8209,7 +8219,7 @@
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B108" s="2" t="n">
         <v>151.088</v>
@@ -8268,7 +8278,7 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B109" s="2" t="n">
         <v>195.927</v>
@@ -8327,7 +8337,7 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B110" s="2" t="n">
         <v>137.5</v>
@@ -8386,7 +8396,7 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B111" s="2" t="n">
         <v>147.884</v>
@@ -8445,7 +8455,7 @@
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B112" s="2" t="n">
         <v>165.367</v>
@@ -8504,7 +8514,7 @@
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B113" s="2" t="n">
         <v>162.335</v>
@@ -8563,7 +8573,7 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B114" s="2" t="n">
         <v>141.117</v>
@@ -8622,7 +8632,7 @@
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B115" s="2" t="n">
         <v>177.058</v>
@@ -8681,7 +8691,7 @@
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B116" s="2" t="n">
         <v>176.84</v>
@@ -8740,7 +8750,7 @@
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B117" s="2" t="n">
         <v>172.897</v>
@@ -8799,7 +8809,7 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B118" s="2" t="n">
         <v>147.548</v>
@@ -8858,7 +8868,7 @@
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B119" s="2" t="n">
         <v>130.463</v>
@@ -8917,7 +8927,7 @@
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B120" s="2" t="n">
         <v>155.54</v>
@@ -8976,7 +8986,7 @@
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B121" s="2" t="n">
         <v>141.833</v>
@@ -9035,7 +9045,7 @@
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B122" s="2" t="n">
         <v>116.669</v>
@@ -9094,7 +9104,7 @@
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B123" s="2" t="n">
         <v>108.482</v>
@@ -9153,7 +9163,7 @@
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B124" s="2" t="n">
         <v>70.196</v>
@@ -9212,7 +9222,7 @@
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B125" s="2" t="n">
         <v>12.585</v>
@@ -9271,7 +9281,7 @@
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B126" s="2" t="n">
         <v>82.176</v>
@@ -9330,7 +9340,7 @@
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B127" s="2" t="n">
         <v>90.948</v>
@@ -9389,7 +9399,7 @@
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B128" s="2" t="n">
         <v>115.216</v>
@@ -9448,7 +9458,7 @@
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B129" s="2" t="n">
         <v>102.731</v>
@@ -9507,7 +9517,7 @@
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B130" s="2" t="n">
         <v>97.709</v>
@@ -9566,7 +9576,7 @@
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B131" s="2" t="n">
         <v>145.1</v>
@@ -9625,7 +9635,7 @@
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B132" s="2" t="n">
         <v>146.632</v>
@@ -9684,7 +9694,7 @@
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B133" s="2" t="n">
         <v>130.831</v>
@@ -9743,7 +9753,7 @@
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B134" s="2" t="n">
         <v>124.937</v>
@@ -9802,7 +9812,7 @@
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B135" s="2" t="n">
         <v>107.334</v>
@@ -9861,7 +9871,7 @@
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B136" s="2" t="n">
         <v>130.274</v>
@@ -9920,7 +9930,7 @@
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B137" s="2" t="n">
         <v>148.013</v>
@@ -9979,7 +9989,7 @@
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B138" s="2" t="n">
         <v>152.032</v>
@@ -10038,7 +10048,7 @@
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B139" s="2" t="n">
         <v>190.652</v>
@@ -10097,7 +10107,7 @@
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B140" s="2" t="n">
         <v>150.607</v>
@@ -10156,7 +10166,7 @@
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B141" s="2" t="n">
         <v>147.473</v>
@@ -10215,7 +10225,7 @@
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B142" s="2" t="n">
         <v>167.818</v>
@@ -10274,7 +10284,7 @@
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B143" s="2" t="n">
         <v>116.992</v>
@@ -10333,7 +10343,7 @@
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B144" s="2" t="n">
         <v>149.271</v>
@@ -10392,7 +10402,7 @@
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B145" s="2" t="n">
         <v>175.795</v>
@@ -10451,7 +10461,7 @@
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B146" s="2" t="n">
         <v>93.974</v>
@@ -10510,7 +10520,7 @@
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B147" s="2" t="n">
         <v>155.567</v>
@@ -10569,7 +10579,7 @@
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B148" s="2" t="n">
         <v>139.789</v>
@@ -10628,7 +10638,7 @@
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B149" s="2" t="n">
         <v>170.022</v>
@@ -10687,7 +10697,7 @@
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B150" s="2" t="n">
         <v>188.16</v>
@@ -10746,7 +10756,7 @@
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B151" s="2" t="n">
         <v>146.259</v>
@@ -10805,7 +10815,7 @@
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B152" s="2" t="n">
         <v>141.609</v>
@@ -10864,7 +10874,7 @@
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B153" s="2" t="n">
         <v>154.726</v>
@@ -10923,7 +10933,7 @@
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B154" s="2" t="n">
         <v>166.859</v>
@@ -10982,7 +10992,7 @@
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B155" s="2" t="n">
         <v>151.186</v>
@@ -11041,7 +11051,7 @@
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B156" s="2" t="n">
         <v>183.115</v>
@@ -11100,7 +11110,7 @@
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B157" s="2" t="n">
         <v>149.612</v>
@@ -11159,7 +11169,7 @@
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B158" s="2" t="n">
         <v>210.371</v>
@@ -11218,7 +11228,7 @@
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B159" s="2" t="n">
         <v>138.999</v>
@@ -11277,7 +11287,7 @@
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B160" s="2" t="n">
         <v>170.199</v>
@@ -11336,7 +11346,7 @@
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B161" s="2" t="n">
         <v>145.096</v>
@@ -11395,7 +11405,7 @@
     </row>
     <row r="162">
       <c r="A162" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B162" s="2" t="n">
         <v>125.404</v>
@@ -11454,7 +11464,7 @@
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B163" s="2" t="n">
         <v>182.956</v>
@@ -11513,7 +11523,7 @@
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B164" s="2" t="n">
         <v>144.35</v>
@@ -11572,7 +11582,7 @@
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B165" s="2" t="n">
         <v>186.728</v>
@@ -11631,7 +11641,7 @@
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B166" s="2" t="n">
         <v>195.217</v>
@@ -11690,7 +11700,7 @@
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B167" s="2" t="n">
         <v>140.332</v>
@@ -11749,7 +11759,7 @@
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B168" s="2" t="n">
         <v>171.765</v>
@@ -11808,7 +11818,7 @@
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B169" s="2" t="n">
         <v>133.409</v>
@@ -11867,7 +11877,7 @@
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B170" s="2" t="n">
         <v>103.697</v>
@@ -11926,7 +11936,7 @@
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B171" s="2" t="n">
         <v>92.041</v>
@@ -11985,7 +11995,7 @@
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B172" s="2" t="n">
         <v>127.362</v>
@@ -12044,7 +12054,7 @@
     </row>
     <row r="173">
       <c r="A173" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B173" s="2" t="n">
         <v>93.3</v>
@@ -12103,7 +12113,7 @@
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B174" s="2" t="n">
         <v>105.036</v>
@@ -12162,7 +12172,7 @@
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B175" s="2" t="n">
         <v>89.278</v>
@@ -12221,7 +12231,7 @@
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B176" s="2" t="n">
         <v>138.624</v>
@@ -12280,7 +12290,7 @@
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B177" s="2" t="n">
         <v>160.941</v>
@@ -12339,7 +12349,7 @@
     </row>
     <row r="178">
       <c r="A178" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B178" s="2" t="n">
         <v>167.52</v>
@@ -12398,7 +12408,7 @@
     </row>
     <row r="179">
       <c r="A179" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B179" s="2" t="n">
         <v>189.966</v>
@@ -12457,7 +12467,7 @@
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B180" s="2" t="n">
         <v>85.931</v>
@@ -12516,7 +12526,7 @@
     </row>
     <row r="181">
       <c r="A181" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B181" s="2" t="n">
         <v>137.012</v>
@@ -12575,7 +12585,7 @@
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B182" s="2" t="n">
         <v>86.319</v>
@@ -12634,7 +12644,7 @@
     </row>
     <row r="183">
       <c r="A183" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B183" s="2" t="n">
         <v>88.329</v>
@@ -12693,7 +12703,7 @@
     </row>
     <row r="184">
       <c r="A184" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B184" s="2" t="n">
         <v>105.774</v>
@@ -12752,7 +12762,7 @@
     </row>
     <row r="185">
       <c r="A185" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B185" s="2" t="n">
         <v>122.552</v>
@@ -12811,7 +12821,7 @@
     </row>
     <row r="186">
       <c r="A186" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B186" s="2" t="n">
         <v>114.562</v>
@@ -12870,7 +12880,7 @@
     </row>
     <row r="187">
       <c r="A187" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B187" s="2" t="n">
         <v>146.96</v>
@@ -12929,7 +12939,7 @@
     </row>
     <row r="188">
       <c r="A188" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B188" s="2" t="n">
         <v>109.831</v>
@@ -12988,7 +12998,7 @@
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B189" s="2" t="n">
         <v>100.383</v>
@@ -13047,7 +13057,7 @@
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B190" s="2" t="n">
         <v>105.128</v>
@@ -13106,7 +13116,7 @@
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B191" s="2" t="n">
         <v>161.202</v>
@@ -13165,7 +13175,7 @@
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B192" s="2" t="n">
         <v>113.804</v>
@@ -13224,7 +13234,7 @@
     </row>
     <row r="193">
       <c r="A193" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B193" s="2" t="n">
         <v>117.461</v>
@@ -13283,7 +13293,7 @@
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B194" s="2" t="n">
         <v>93.932</v>
@@ -13342,7 +13352,7 @@
     </row>
     <row r="195">
       <c r="A195" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B195" s="2" t="n">
         <v>99.895</v>
@@ -13401,7 +13411,7 @@
     </row>
     <row r="196">
       <c r="A196" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B196" s="2" t="n">
         <v>112.034</v>
@@ -13460,7 +13470,7 @@
     </row>
     <row r="197">
       <c r="A197" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B197" s="2" t="n">
         <v>113.545</v>
@@ -13519,7 +13529,7 @@
     </row>
     <row r="198">
       <c r="A198" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B198" s="2"/>
       <c r="C198" s="3" t="n">
@@ -13552,7 +13562,7 @@
     </row>
     <row r="199">
       <c r="A199" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B199" s="2"/>
       <c r="C199" s="3" t="n">
@@ -13585,7 +13595,7 @@
     </row>
     <row r="200">
       <c r="A200" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B200" s="2"/>
       <c r="C200" s="3" t="n">
@@ -13618,7 +13628,7 @@
     </row>
     <row r="201">
       <c r="A201" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B201" s="2"/>
       <c r="C201" s="3" t="n">
@@ -13651,7 +13661,7 @@
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B202" s="2"/>
       <c r="C202" s="3" t="n">
@@ -13684,7 +13694,7 @@
     </row>
     <row r="203">
       <c r="A203" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B203" s="2"/>
       <c r="C203" s="3" t="n">
@@ -13717,7 +13727,7 @@
     </row>
     <row r="204">
       <c r="A204" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B204" s="2"/>
       <c r="C204" s="3" t="n">
@@ -13750,7 +13760,7 @@
     </row>
     <row r="205">
       <c r="A205" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B205" s="2"/>
       <c r="C205" s="3" t="n">
@@ -13783,7 +13793,7 @@
     </row>
     <row r="206">
       <c r="A206" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B206" s="2"/>
       <c r="C206" s="3" t="n">
@@ -13816,7 +13826,7 @@
     </row>
     <row r="207">
       <c r="A207" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B207" s="2"/>
       <c r="C207" s="3" t="n">
@@ -13849,7 +13859,7 @@
     </row>
     <row r="208">
       <c r="A208" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B208" s="2"/>
       <c r="C208" s="3" t="n">
@@ -13882,7 +13892,7 @@
     </row>
     <row r="209">
       <c r="A209" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B209" s="2"/>
       <c r="C209" s="3" t="n">
@@ -13915,7 +13925,7 @@
     </row>
     <row r="210">
       <c r="A210" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B210" s="2"/>
       <c r="C210" s="3"/>
@@ -13938,7 +13948,7 @@
     </row>
     <row r="211">
       <c r="A211" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B211" s="2"/>
       <c r="C211" s="3"/>
@@ -13961,7 +13971,7 @@
     </row>
     <row r="212">
       <c r="A212" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B212" s="2"/>
       <c r="C212" s="3"/>
@@ -13984,7 +13994,7 @@
     </row>
     <row r="213">
       <c r="A213" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B213" s="2"/>
       <c r="C213" s="3"/>
@@ -14007,7 +14017,7 @@
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B214" s="2"/>
       <c r="C214" s="3"/>
@@ -14030,7 +14040,7 @@
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B215" s="2"/>
       <c r="C215" s="3"/>
@@ -14053,7 +14063,7 @@
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B216" s="2"/>
       <c r="C216" s="3"/>
@@ -14076,7 +14086,7 @@
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B217" s="2"/>
       <c r="C217" s="3"/>
@@ -14099,7 +14109,7 @@
     </row>
     <row r="218">
       <c r="A218" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B218" s="2"/>
       <c r="C218" s="3"/>
@@ -14122,7 +14132,7 @@
     </row>
     <row r="219">
       <c r="A219" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B219" s="2"/>
       <c r="C219" s="3"/>
@@ -14145,7 +14155,7 @@
     </row>
     <row r="220">
       <c r="A220" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B220" s="2"/>
       <c r="C220" s="3"/>
@@ -14168,7 +14178,7 @@
     </row>
     <row r="221">
       <c r="A221" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B221" s="2"/>
       <c r="C221" s="3"/>
@@ -14191,7 +14201,7 @@
     </row>
     <row r="222">
       <c r="A222" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B222" s="2"/>
       <c r="C222" s="3"/>
@@ -14214,7 +14224,7 @@
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B223" s="2"/>
       <c r="C223" s="3"/>
@@ -14237,7 +14247,7 @@
     </row>
     <row r="224">
       <c r="A224" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B224" s="2"/>
       <c r="C224" s="3"/>
@@ -14260,7 +14270,7 @@
     </row>
     <row r="225">
       <c r="A225" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B225" s="2"/>
       <c r="C225" s="3"/>
@@ -14283,7 +14293,7 @@
     </row>
     <row r="226">
       <c r="A226" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B226" s="2"/>
       <c r="C226" s="3"/>
@@ -14306,7 +14316,7 @@
     </row>
     <row r="227">
       <c r="A227" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B227" s="2"/>
       <c r="C227" s="3"/>
@@ -14329,7 +14339,7 @@
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B228" s="2"/>
       <c r="C228" s="3"/>
@@ -14352,7 +14362,7 @@
     </row>
     <row r="229">
       <c r="A229" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B229" s="2"/>
       <c r="C229" s="3"/>
@@ -14375,7 +14385,7 @@
     </row>
     <row r="230">
       <c r="A230" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B230" s="2"/>
       <c r="C230" s="3"/>
@@ -14398,7 +14408,7 @@
     </row>
     <row r="231">
       <c r="A231" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B231" s="2"/>
       <c r="C231" s="3"/>
@@ -14421,7 +14431,7 @@
     </row>
     <row r="232">
       <c r="A232" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B232" s="2"/>
       <c r="C232" s="3"/>
@@ -14444,7 +14454,7 @@
     </row>
     <row r="233">
       <c r="A233" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B233" s="2"/>
       <c r="C233" s="3"/>
@@ -14467,7 +14477,7 @@
     </row>
     <row r="234">
       <c r="A234" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B234" s="2"/>
       <c r="C234" s="3"/>
@@ -14490,7 +14500,7 @@
     </row>
     <row r="235">
       <c r="A235" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B235" s="2"/>
       <c r="C235" s="3"/>
@@ -14513,7 +14523,7 @@
     </row>
     <row r="236">
       <c r="A236" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B236" s="2"/>
       <c r="C236" s="3"/>
@@ -14536,7 +14546,7 @@
     </row>
     <row r="237">
       <c r="A237" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B237" s="2"/>
       <c r="C237" s="3"/>
@@ -14559,7 +14569,7 @@
     </row>
     <row r="238">
       <c r="A238" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B238" s="2"/>
       <c r="C238" s="3"/>
@@ -14582,7 +14592,7 @@
     </row>
     <row r="239">
       <c r="A239" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B239" s="2"/>
       <c r="C239" s="3"/>
@@ -14605,7 +14615,7 @@
     </row>
     <row r="240">
       <c r="A240" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B240" s="2"/>
       <c r="C240" s="3"/>
@@ -14628,7 +14638,7 @@
     </row>
     <row r="241">
       <c r="A241" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B241" s="2"/>
       <c r="C241" s="3"/>
@@ -14651,7 +14661,7 @@
     </row>
     <row r="242">
       <c r="A242" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B242" s="2"/>
       <c r="C242" s="3"/>
@@ -14674,7 +14684,7 @@
     </row>
     <row r="243">
       <c r="A243" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B243" s="2"/>
       <c r="C243" s="3"/>
@@ -14697,7 +14707,7 @@
     </row>
     <row r="244">
       <c r="A244" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B244" s="2"/>
       <c r="C244" s="3"/>
@@ -14720,7 +14730,7 @@
     </row>
     <row r="245">
       <c r="A245" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B245" s="2"/>
       <c r="C245" s="3"/>
@@ -14743,7 +14753,7 @@
     </row>
     <row r="246">
       <c r="A246" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B246" s="2"/>
       <c r="C246" s="3"/>
@@ -14766,7 +14776,7 @@
     </row>
     <row r="247">
       <c r="A247" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B247" s="2"/>
       <c r="C247" s="3"/>
@@ -14789,7 +14799,7 @@
     </row>
     <row r="248">
       <c r="A248" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B248" s="2"/>
       <c r="C248" s="3"/>
@@ -14812,7 +14822,7 @@
     </row>
     <row r="249">
       <c r="A249" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B249" s="2"/>
       <c r="C249" s="3"/>
@@ -14835,7 +14845,7 @@
     </row>
     <row r="250">
       <c r="A250" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B250" s="2"/>
       <c r="C250" s="3"/>
@@ -14858,7 +14868,7 @@
     </row>
     <row r="251">
       <c r="A251" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B251" s="2"/>
       <c r="C251" s="3"/>
@@ -14881,7 +14891,7 @@
     </row>
     <row r="252">
       <c r="A252" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B252" s="2"/>
       <c r="C252" s="3"/>
@@ -14904,7 +14914,7 @@
     </row>
     <row r="253">
       <c r="A253" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B253" s="2"/>
       <c r="C253" s="3"/>
@@ -14938,97 +14948,97 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
     </row>
   </sheetData>
@@ -15052,7 +15062,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -15062,13 +15072,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>-0.129800873098031</v>
@@ -15076,7 +15086,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>-0.118350302837531</v>
@@ -15084,7 +15094,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>-0.0559726123126038</v>
@@ -15092,7 +15102,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>-0.0236657333528303</v>
@@ -15100,7 +15110,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>0.0489194470114575</v>
@@ -15108,7 +15118,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>0.124295227370116</v>
@@ -15116,7 +15126,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>0.119404710344242</v>
@@ -15124,7 +15134,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>0.176591651987928</v>
@@ -15132,7 +15142,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>0.341562757767561</v>
@@ -15140,7 +15150,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>0.383864490777403</v>
@@ -15148,7 +15158,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>0.292872297049826</v>
@@ -15156,7 +15166,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>0.28544176945417</v>
@@ -15164,7 +15174,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>0.285974000422875</v>
@@ -15172,7 +15182,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>0.179659724492369</v>
@@ -15180,7 +15190,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>0.0311476927942055</v>
@@ -15188,7 +15198,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>-0.114994337057583</v>
@@ -15196,7 +15206,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>-0.184230706536227</v>
@@ -15204,7 +15214,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>-0.136627224919718</v>
@@ -15212,7 +15222,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>-0.104097604842097</v>

</xml_diff>

<commit_message>
Corrida | SFE-SUPT | 2026-07-01 09:47:56.666525
</commit_message>
<xml_diff>
--- a/indicadores/SFE-SUPT_out.xlsx
+++ b/indicadores/SFE-SUPT_out.xlsx
@@ -29,7 +29,7 @@
     <t xml:space="preserve">Unidad de medida</t>
   </si>
   <si>
-    <t xml:space="preserve">Miles de m2</t>
+    <t xml:space="preserve">Miles de m²</t>
   </si>
   <si>
     <t xml:space="preserve">Ajuste estacional</t>
@@ -15289,237 +15289,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C5B9F2161CEE1040BBC03CB11300495F" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a7cec21613a3259523bdab11a1e26aca">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5dd4176-d247-4204-85b8-921214f3ccea" xmlns:ns3="359b39ce-e1f9-4933-8424-33b611e6fdcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="68943c349d3a016936c8f8cb3335004b" ns2:_="" ns3:_="">
-    <xsd:import namespace="b5dd4176-d247-4204-85b8-921214f3ccea"/>
-    <xsd:import namespace="359b39ce-e1f9-4933-8424-33b611e6fdcd"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5dd4176-d247-4204-85b8-921214f3ccea" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="01529062-7a8b-4d76-943d-e0db5644ee6d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="359b39ce-e1f9-4933-8424-33b611e6fdcd" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c9b73259-0823-4f05-8927-4a40ee49fbe1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="359b39ce-e1f9-4933-8424-33b611e6fdcd">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CBD7371C-2D29-45E4-8B9D-05FA25146A8B}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EBDDBD40-5A76-4A99-81A5-68A396BAAD21}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{501F7CAF-F7C5-4D49-A278-19ECAA0E4237}"/>
 </file>
</xml_diff>